<commit_message>
feat: reorganiza organograma com layout classico - fileira horizontal no 1o nivel e subordinacoes abertas horizontalmente
</commit_message>
<xml_diff>
--- a/Relatorio_IFRS_Final_v11.xlsx
+++ b/Relatorio_IFRS_Final_v11.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcraf\codes\regimento-vacaria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085204FC-5CF4-4773-B1A1-365F4C63986E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCFB0B5C-F678-4801-A28A-F0DEFAA9D0CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setores_Comparativo" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="218">
   <si>
     <t>Setor</t>
   </si>
@@ -254,9 +254,6 @@
 VIII – recepcionar os visitantes do Gabinete.</t>
   </si>
   <si>
-    <t>Setor de Comunicação</t>
-  </si>
-  <si>
     <t>Art. 9. O Setor de Comunicação é responsável pela comunicação do IFRS Campus Vacaria com
 seus públicos.
 Parágrafo único. As atividades do Setor de Comunicação serão exercidas por equipe composta
@@ -284,172 +281,6 @@
 XI. Integrar a Comissão responsável pela edição e publicação do Boletim de Serviços;
 XII. Desempenhar outras atividades correlatas ao setor de comunicação, ao cargo ou definidas
 pela legislação e/ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
-    <t>--- Resolução Nº 14 - Regimento Complementar do Campus Canoas - Ano 2018 ---
-Art. 22º O setor de comunicação, concebido como sistêmico dentro da
-unidade por congregar ações que integram as áreas do ensino, da pesquisa e
-da extensão, está subordinado à direção-geral, e congrega, minimamente os
-cargos de jornalista e de técnico em audiovisual.
-Art. 23º Compete ao jornalista desempenhar as seguintes ações:
-I. Promover a divulgação jornalística de eventos e atividades de
-cunho institucional por meio de diferentes veículos de comunicação,
-estabelecendo um canal permanente entre os veículos e o Campus;
-II. Estabelecer contato com os veículos de comunicação e promover
-a divulgação das ações da unidade, no que tange à parte jornalística, na
-modalidade de sugestão de pauta (releases);
-III. Trabalhar na criação e na constante manutenção de publicações
-de cunho jornalístico em nível de campus, que venham ao encontro das
-políticas de comunicação do IFRS;
-IV. Implementar, em nível de campus, as ações provenientes da
-política de comunicação, elaborada pela Diretoria de Comunicação do IFRS,
-em consonância com a realidade de cada unidade;
-V. Estabelecer critérios de fixação e controle de cartazes, faixas,
-murais e outras formas de divulgação no Campus;
-VI. Promover a manutenção dos diversos tipos de mídia criados pelo
-IFRS;
-VII. Promover o diálogo dos diversos veículos de comunicação com o
-Campus, no que tange as divulgações de cunho jornalístico;
-VIII. Participar da Comissão Permanente de Formatura, como membro
-nato, de acordo com normativas estabelecidas pelo IFRS;
-IX. Participar da Comissão Permanente de Seleção do Processo
-Seletivo, de acordo com a Política de Ingresso Discente;
-Regimento Complementar do IFRS – Campus Canoas – Página 19 de 41
-X. Participar da Comissão de elaboração e formatação do Boletim
-de Serviço da unidade.
-Art. 24º Compete ao Técnico em Audiovisual desempenhar as seguintes
-ações:
-I. Produzir e editar filmes institucionais e matérias jornalísticas em
-áudio e vídeo, em conjunto com o jornalista ou outros profissionais da
-Comunicação;
-II. Atuar com equipamentos audiovisuais (alto-falantes, microfones,
-amplificadores, projetores e similares);
-III. Manejar equipamentos audiovisuais, registrando som, foto e
-vídeo nas atividades institucionais, didáticas, de pesquisa e extensão;
-IV. Utilizar recursos multimídia na edição de imagens e sons;
-V. Testar a instalação, fazendo as conexões e os ajustes
-convenientes;
-VI. Manter-se atualizado sobre as tecnologias audiovisuais e outras,
-sugerindo e coordenando a aquisição de novos equipamentos e recursos;
-VII. Zelar pelo cumprimento das normas e legislações de uso de
-imagem;
-VIII. Manter e conservar os equipamentos;
-IX. Encaminhar, quando necessário, os equipamentos para
-manutenção, auxiliando na obtenção de orçamentos;
-X. Controlar a circulação dos equipamentos, registrando a
-movimentação em fichário apropriado;
-XI. Manter organizado e atualizado os arquivos de imagens
-fotográficas e cinematográficas, bem como os de áudio;
-XII. Executar outras tarefas de mesma natureza e nível de
-complexidade, associadas ao ambiente organizacional;
-XIII. Desempenhar outras atividades afins ou previstas na legislação
-vigente.
---- Resolução Nº 20 - Regimento Complementar do Campus Erechim - Ano 2024 ---
-Art. 18º O setor de comunicação, concebido como sistêmico dentro da unidade por
-congregar ações que integram as áreas do ensino, da pesquisa e da extensão,
-está subordinado à direção-geral.
-Art. 19º Compete ao Setor de Comunicação desempenhar as seguintes ações:
-I. Promover a divulgação jornalística de eventos e atividades de cunho
-institucional por meio de diferentes veículos de comunicação, estabelecendo
-um canal permanente entre os veículos e o Campus;
-II. Estabelecer contato com os veículos de comunicação e promover a
-divulgação das ações da unidade, no que tange à parte jornalística, na
-modalidade de sugestão de pauta (releases);
-III. Trabalhar na criação e na constante manutenção de publicações de cunho
-jornalístico em nível de campus, que venham ao encontro das políticas de
-comunicação do IFRS;
-IV. Implementar, em nível de campus, as ações provenientes da política de
-comunicação, elaborada pela Diretoria de Comunicação do IFRS, em
-consonância com a realidade de cada unidade;
-V. Estabelecer critérios de fixação e controle de cartazes, faixas, murais e
-outras formas de divulgação no Campus;
-VI. Promover a manutenção dos diversos tipos de mídia criados pelo IFRS;
-VII. Promover o diálogo dos diversos veículos de comunicação com o campus, no
-que tange as divulgações de cunho jornalístico;
-VIII. Participar da Comissão Permanente de Formatura, como membro nato, de
-acordo com normativas estabelecidas pelo IFRS;
-IX. Participar da Comissão Permanente de Seleção do Processo Seletivo, de
-acordo com a Política de Ingresso Discente.
-Da Coordenação de Gestão de Pessoas
-Art. 20º À Coordenação de Gestão de Pessoas, subordinada à Direção Geral,
-compete:
-I. Acompanhar e aplicar programas de capacitação visando ao
-aperfeiçoamento funcional do servidor;
-II. Atualizar periodicamente o cadastro dos servidores;
-III. Acompanhar e formalizar a movimentação dos servidores;
-IV. Atualizar permanentemente o quadro de lotação;
-V. Organizar e acompanhar o processo de estágio probatório;
-VI. Gerenciar a distribuição dos benefícios sociais aos servidores;
-VII. Receber e encaminhar as demandas para provimento de cargos;
-VIII. Orientar e acompanhar as progressões funcionais dos servidores;
-IX. Desenvolver programas que facilitem a integração de novos servidores;
-X. Organizar, controlare manter atualizados os arquivos de documentos e
-dados cadastrais dos servidores do Campus;
-XI. Interpretar e prestar esclarecimentos sobre a legislação, normas, fluxos e
-processos de pessoal;
-XII. Exercer atividades relacionadas à admissão, desligamento,
-aperfeiçoamento, lotação, pagamento e cadastro de servidores;
-XIII. Efetivar os devidos registros e operações do processamento da folha de
-pagamento dos servidores;
-XIV. Emitir documentos oficiais com base nos registros constantes no cadastro
-geral dos servidores;
-XV. Orientar as chefias imediatas quanto ao controle de frequência, conforme
-legislação vigente;
-XVI. Prestar informações à comunidade sobre assuntos de sua competência;
-XVII. Promover o controle de lotação dos cargos de direção e funções
-gratificadas, bem como elaborar os atos próprios;
-XVIII. Oferecer subsídios para o planejamento orçamentário de recursos humanos;
-XIX. Elaborar e controlar processos de inatividade e pensões;
-XX. Preparar os atos de processamento e controle das alterações funcionais;
-XXI. Executar e avaliar projetos e ações que contribuam para a qualidade de vida
-dos servidores;
-XXII. Elaborar e realizar as publicações dos atos de pessoal no Diário Oficial da
-União e no Boletim de Serviço Interno.
-XXIII. Realizar em conjunto com a COA (Comissão de Organização e
-Acompanhamento) e a gestão, o relatório anual das ações de
-desenvolvimento de pessoas do Campus.
-XXIV. Receber as demandas para contratação de estagiários, realizar processos
-seletivos, inclusão na folha de pagamento, controle das avaliações
-semestrais, prazos de renovação, e rescisões.
---- Resolução Nº 23 - Regimento Complementar do Campus Ibirubá - Ano 2025 ---
-Art.28 As atividades da Assessoria de Comunicação envolvem:
-I. Planejar e executar as ações de comunicação, em consonância com
-as diretrizes da Secretaria de Comunicação do Ministério da
-Educação;
-II. Reunir para elaborar pauta, coleta e organização de informações,
-assim como a posterior elaboração de matérias referentes ao
-Campus;
-III. Atualizar o Portal e as redes sociais do Campus;
-IV. Registrar reuniões e eventos institucionais do Campus por meio de
-ferramentas de áudio e/ou imagem, de acordo com o planejamento
-estratégico da área;
-V. Assistir ao Diretor Geral na coordenação de programas, projetos e
-ações de divulgação do Campus nos assuntos relativos à imprensa,
-marketing e integração social com a comunidade.
-Da Coordenação de Gestão de Pessoas
-Art.29 À Coordenação de Gestão de Pessoas, subordinada à Direção Geral,
-compete:
-I. Organizar e manter registros atualizados sobre a vida funcional dos
-servidores;
-II. Atualizar permanentemente o quadro de localização dos servidores;
-III. Organizar e acompanhar os processos de estágio probatório;
-IV. Receber e encaminhar as demandas para provimento de cargos;
-V. Orientar sobre as progressões funcionais dos servidores;
-VI. Analisar os requerimentos de sua competência, atribuída pela DGP;
-VII. Protocolar e tramitar os processos de sua competência;
-VIII. Efetivar os devidos registros e operações do processamento da folha
-de pagamento dos servidores;
-IX. Emitir documentos oficiais com base nos registros constantes no
-cadastro geral dos servidores;
-X. Prestar informações sobre assuntos de sua competência;
-XI. Receber e conduzir as demandas para contratação de estagiários,
-professores substitutos e professores visitantes, realizando a abertura
-de editais para seleção, o processo de contratação, os termos
-aditivos, alterações, controle de prazos, rescisões e publicações dos
-13
-atos no Diário Oficial;
-XII. Desempenhar outras atividades correlatas à Coordenadoria, ao cargo
-ou definidas pela legislação e/ou atribuídas pelo superior hierárquico.</t>
   </si>
   <si>
     <t>Coordenadoria de Gestão de Pessoas</t>
@@ -1979,45 +1810,6 @@
     <t>Coordenadoria de Ensino</t>
   </si>
   <si>
-    <t>Art. 40. A Coordenadoria de Ensino, de forma articulada com a Diretoria de Ensino é o órgão
-responsável por planejar, coordenar, executar, acompanhar e avaliar as políticas educacionais e
-diretrizes de ensino no Campus.
-Art. 41. As atividades da Coordenadoria de Ensino serão exercidas por um servidor efetivo do
-quadro de pessoal do IFRS designado pelo(a) Diretor(a) Geral do Campus.
-Art. 42. À Coordenadoria de Ensino, subordinada à Diretoria de Ensino, compete as seguintes
-atribuições:
-I. Colaborar com o planejamento e constante aperfeiçoamento da Coordenadoria, visando
-atender as demandas de ensino, pesquisa, extensão e gestão existentes na Instituição,
-racionalizando o uso dos recursos e equipamentos;
-II. Planejar, acompanhar e avaliar a proposta pedagógica institucional, nos diferentes níveis
-de ensino oferecidos aos discentes;
-III. Acompanhar o planejamento e a execução dos processos de ensino e aprendizagem;
-IV. Acompanhar a elaboração das propostas pedagógicas;
-V. Encaminhar para aprovação do Conselho de Campus os projetos pedagógicos de cursos
-de Ensino Médio;
-VI. Encaminhar para aprovação no Conselho de Campus as normas de utilização dos espaços
-destinados ao ensino;
-VII. Supervisionar os diários de classe dos componentes curriculares de todos os níveis de
-ensino ofertados pelo campus, junto aos professores e acompanhar sua manutenção, bem como
-os registros de rendimento acadêmico dos estudantes;
-VIII. Elaborar e coordenar a publicação de editais relativos a monitorias, promovendo a gestão
-administrativa, incluindo inscrições, controle de frequência e certificação;
-IX. Elaborar quadro de horários;
-X. Organizar os conselhos de classe;
-XI. Propor atividades de capacitação aos Docentes e Técnicos Administrativos em Educação;
-XII. Responder pelo Diretor de Ensino na sua ausência ou impedimento;
-XIII. Desempenhar outras atividades correlatas à Coordenadoria de Ensino, ao cargo ou
-14
-definidas pela legislação e/ou atribuídas pelo superior hierárquico.
-Das Coorde nadorias de Cursos
-Art. 43. As atividades das Coordenadorias de Cursos, subordinadas à Coordenadoria de Ensino,
-serão exercidas por servidores efetivos do quadro de pessoal do IFRS, eleitos pelo respectivo
-colegiado de curso e nomeados pelo(a) Diretor(a) Geral de Campus.
-Parágrafo único. Às Coordenadorias de Cursos compete a gestão didático-pedagógica dos cursos,
-tendo suas atribuições regulamentadas em Regimento próprio aprovado pelo Conselho Superior
-do IFRS.</t>
-  </si>
-  <si>
     <t>--- Resolução Nº 14 - Regimento Complementar do Campus Canoas - Ano 2018 ---
 Art. 9º À Coordenadoria de Ensino, subordinada à Direção de Ensino,
 compete:
@@ -2136,181 +1928,6 @@
 X. Implementar programas de tecnologia educacional;
 XI. Desempenhar outras atividades correlatas ao setor, ao cargo ou definidas pela legislação
 e/ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
-    <t>--- Resolução Nº 034 - Regimento Complementar do Campus Bento Gonçalves - Ano 2024 ---
-Art. 57. A Diretoria de Ensino é dirigida por um(a) Diretor(a) de Ensino nomeado pelo(a)
-Diretor(a)-geral.
-Parágrafo único. As competências da Gestão de Ensino estão previstas no art. 23 da
-Resolução Consup IFRS nº 054, de 15/08/2017 (Regimento dos Campi do IFRS).
-Art. 58. A Diretoria de Ensino é composta pela Coordenadoria de Ensino Médio e
-Educação Profissional, Coordenadoria de Ensino de Graduação, Coordenadoria de
-Assuntos Estudantis (CAE), Coordenadoria de Registros Acadêmicos (CRA),
-Coordenadoria Pedagógica, Seção de Biblioteca, Seção de Estágios, Núcleo de Ensino a
-Distância (NEAD), Núcleo de Atendimento a Pessoas com Necessidades Educacionais
-Específicas (NAPNE) e Núcleos de Integração do Ensino, Pesquisa e Extensão (NIEPEs).
-17
---- Resolução Nº 23 - Regimento Complementar do Campus Ibirubá - Ano 2025 ---
-Art.56 As atividades de Gestão de Ensino serão exercidas por um servidor efetivo
-do quadro de pessoal do IFRS, designado pelo Diretor-geral do campus.
-Parágrafo único. As competências da Gestão de Ensino estão previstas no
-Regimento Geral dos Campi do IFRS.
-Da Coordenação de Ensino
-Art.57 A Coordenadoria de Ensino é um órgão executivo do Campus, subordinado
-à Gestão de Ensino e desempenhado por um coordenador de Ensino,
-nomeado pelo Diretor Geral.
-Art.58 Compete à Coordenadoria de Ensino:
-I. Planejar, organizar e divulgar ações relativas às atividades de
-ensino, em todos os níveis de Ensino;
-II. Elaborar e acompanhar, juntamente com a Comissão de Avaliação e
-Gestão do Ensino- CAGE, o calendário acadêmico para todos os
-níveis de Ensino;
-III. Garantir espaços para a realização de atividades de Formação
-Continuada dos servidores, realizando, pelo menos, uma atividade no
-início do ano letivo, prevendo a participação dos Núcleos de Ações
-Afirmativas;
-IV. Promover ações que visam ao compartilhamento de conhecimentos e
-à integração da comunidade acadêmica, tais como: Seminários,
-Mostra de Trabalhos, Oficinas e Simpósios;
-V. Planejar, organizar e acompanhar, juntamente com a Direção de
-Ensino, Setor Pedagógico, Assistência Estudantil, Coordenação de
-Curso e docentes, reuniões de acompanhamento da rotina escolar;
-VI. Acompanhar, juntamente com a Direção de Ensino, Setor
-Pedagógico, Assistência Estudantil, Coordenação de Curso, docentes
-e representação estudantil, reuniões de Conselhos de Classe;
-VII. Viabilizar a promoção de ações e espaços formativos aos Núcleos do
-IFRS;
-VIII. Gerenciar , juntamente com a Comissão de Avaliação e Gestão do
-Ensino- CAGE, o planejamento, a divulgação, a execução e avaliação
-dos Editais vinculados ao Ensino.
-IX. Solicitar, junto à Coordenadoria de Administração e Planejamento, o
-empenho e pagamento de recursos financeiros e bolsas relativos aos
-Editais de Ensino.
-X. Mediar, juntamente com a Comissão de Avaliação e Gestão do
-Ensino- CAGE, a prestação de contas de Projetos de Ensino
-contemplados com fomento;
-27
-XI. Certificar coordenadores, colaboradores e estudantes vinculados ao
-desenvolvimento das atividades previstas nos projetos de Ensino
-XII. Coordenar, acompanhar e orientar docentes sobre a rotina
-acadêmica;
-XIII. Coordenar, acompanhar e avaliar o desenvolvimento do processo de
-ensino-aprendizagem;
-XIV. Operacionalizar as ações previstas na política de desenvolvimento
-Institucional para o Ensino;
-XV. Viabilizar Ações de Permanência e Êxito;
-XVI. Acompanhar, juntamente com a Direção de Ensino, Coordenação de
-Curso e Setor Pedagógico a elaboração e atualização dos Projetos
-Pedagógicos dos Cursos;
-XVII. Acompanhar a elaboração e o arquivamento de planos de ensino e
-diários de classe;
-XVIII. Acompanhar o andamento da Progressão Parcial dos cursos do
-Ensino Médio Integrado;
-XIX. Acompanhar a elaboração dos horários dos cursos regulares
-ofertados no Campus juntamente com os Coordenadores de Curso;
-XX. Verificar e emitir atestados de docência;
-XXI. Analisar e deferir requerimentos acerca de justificativas e/ou abono de
-faltas, bem como dos exercícios domiciliares dos estudantes.
-XXII. Gerenciar sistemas, tais como Site do Ensino, Formulários de
-emissão de atestados de naturezas diversas e reserva de
-laboratórios;
-XXIII. Acompanhar as solicitações de Viagem de estudos e/ou viagens
-técnicas junto às Coordenações de Curso;
-XXIV. Analisar e homologar o registro de frequência dos servidores de sua
-competência.
-Do Setor Pedagógico
-Art.59 O Setor Pedagógico tem a função de atuar de forma integrada no
-acompanhamento, na assessoria e na mediação do trabalho pedagógico,
-articulando a ação educativa à Proposta Pedagógica da Instituição,
-viabilizando o trabalho coletivo, contribuindo para a qualificação das relações
-no processo educativo, bem como na formação humana, técnica e científica.
-Art.60 São atribuições da equipe de trabalho:
-I. Coordenar, acompanhar e orientar o planejamento das atividades
-pedagógicas;
-II. Participar da elaboração, execução e avaliação do Projeto
-Pedagógico Institucional e Projetos Pedagógicos dos Cursos;
-III. Acompanhar e mediar as práticas pedagógicas no que se refere ao
-processo ensino-aprendizagem;
-IV. Mediar a elaboração, a execução e o arquivamento dos planos de
-ensino em todos os níveis de ensino;
-V. Orientar e monitorar a finalização e o arquivamento dos diários de
-classe em todos os níveis de ensino;
-28
-VI. Acompanhar a elaboração dos programas de adaptação de currículo,
-atividades de reforço escolar e estudos de recuperação;
-VII. Discutir, propor e analisar resultados da ação pedagógica, visando à
-construção coletiva de alternativas para o êxito do processo
-ensino-aprendizagem e à promoção do desenvolvimento integral do
-educando;
-VIII. Acompanhar as relações entre instituição e família dos estudantes,
-através de encontros individuais e coletivos, tendo em vista a
-construção conjunta de propostas que levem a uma melhoria do
-processo ensino-aprendizagem;
-IX. Elaborar, juntamente com as Coordenações de Curso, os horários dos
-cursos regulares ofertados no Campus;
-X. Realizar o cômputo e encaminhar à Coordenadoria de Registros
-Acadêmicos a carga horária dos componentes curriculares
-colegiados;
-XI. Informar ao Núcleo de Educação a Distância (NEAD) do campus a
-relação de docentes e componentes curriculares para cadastramento
-no Ambiente Virtual de Ensino e Aprendizagem.
-XII. Organizar e orientar ações relativas à Progressão Parcial;
-XIII. Acompanhar, juntamente com a Direção/ Coordenação de Ensino,
-Assistência Estudantil, Coordenação de Curso, docentes e
-representação estudantil, reuniões de Conselhos de Classe;
-XIV. Acompanhar substituições e reposições de aulas dos componentes
-curriculares por motivos previstos em legislação;
-XV. Desempenhar outras atividades correlatas ou definidas pela
-legislação, atribuídas pelo superior hierárquico.
-Das Coordenações de Cursos
-Art.61 Os Coordenadores de Cursos Técnicos e Superiores, subordinados à
-Direção de Ensino, são responsáveis pela gestão didático-pedagógica dos
-cursos. Esses devem fazer parte do quadro efetivo do IFRS - Campus
-Ibirubá e atuar no respectivo Curso, sendo eleitos pelos seus pares.
-Art.62 As competências e atribuições dos Coordenadores de Cursos estão
-descritas na seguinte Resolução: Atribuições dos Coordenadores dos Cursos
-Técnicos, Superiores e de Pós-Graduação Stricto Sensu e Lato Sensu do
-Instituto Federal de Educação, Ciência e Tecnologia do Rio Grande do Sul
-(IFRS), aprovada pelo Conselho Superior do IFRS.
-Parágrafo único. O mandato do Coordenador de curso será de dois anos, permitida
-uma recondução pelo mesmo período.
-29
-Da Coordenação de Registros Acadêmicos
-Art.63 A Coordenadoria de registros acadêmicos, vinculado à Direção de Ensino,
-compete:
-I. Manter atualizadas as informações relacionadas ao quadro discente,
-para controle Institucional e para alimentar o banco de dados dos
-sistemas de informações gerenciais do Ministério da Educação e do
-Campus;
-II. Analisar a vida acadêmica de cada discente e elaborar Diplomas e
-Históricos;
-III. Coordenar e executar o processo de renovação, efetivação de
-matrículas, elaboração de atestados de frequência, pedidos de
-transferência e trancamento de matrícula, providência de lista de
-chamada provisória, diários de classe, boletins escolares,
-requerimentos e outros registros relativos ao corpo discente;
-IV. Recebimento, encaminhamento e lançamento de faltas justificadas,
-abonadas, Exercícios Domiciliares e atividades complementares;
-V. Lançamento e atualização de turmas e horários de aula no sistema
-acadêmico;
-VI. Fornecer, sempre que solicitado, documentação sobre os cursos e
-sobre a vida acadêmica do aluno, obedecendo a legislação vigente;
-VII. Elaboração e coordenação de editais de aproveitamento de estudos,
-certificação de conhecimento, ingresso por transferência, diplomados
-e aluno especial;
-VIII. Receber e encaminhar os pedidos de aproveitamento de estudos e de
-certificação de conhecimentos;
-IX. Verificar e analisar a situação de regularidade dos estudantes, e
-realizar o trancamento ou desligamento de acordo com as orientações
-pré estabelecidas na organização didática institucional;
-X. Gerenciamento e controle das informações relativas ao seguro dos
-estudantes
-XI. Gerenciamento de informações e alimentação de sistemas do
-governo, de responsabilidade do auxiliar institucional;
-XII. Atendimento às demandas gerais do público externo e interno.
-XIII. Zelar pelo sigilo das informações da sua competência;
-XIV. Desempenhar outras atividades correlatas ou definidas pela
-legislação, atribuídas pelo superior hierárquico.</t>
   </si>
   <si>
     <t>Setor de Laboratórios</t>
@@ -2968,126 +2585,6 @@
     <t>Origem</t>
   </si>
   <si>
-    <t>Auditoria Interna</t>
-  </si>
-  <si>
-    <t>Resolução Nº 034 - Regimento Complementar do Campus Bento Gonçalves - Ano 2024</t>
-  </si>
-  <si>
-    <t>Coordenadoria de Ensino Médio e Educação Profissional</t>
-  </si>
-  <si>
-    <t>Art. 59. As atividades da Coordenadoria de Ensino Médio e Educação Profissional serão
-exercidas por um servidor efetivo do quadro de pessoal do IFRS designado pelo(a)
-Diretor(a)-geral do Campus.
-Art. 60. Compete à Coordenadoria de Ensino Médio e Educação Profissional as seguintes
-atribuições:
-I - colaborar com o planejamento e constante aperfeiçoamento da Coordenadoria,
-visando atender as demandas de ensino, pesquisa, extensão e gestão existentes na
-Instituição, racionalizando o uso dos recursos e equipamentos;
-II - elaborar o relatório anual das atividades da Coordenadoria;
-III - planejar o processo de ensino e aprendizagem nos seus aspectos quantitativos e
-qualitativos, com o objetivo de aprimorar e acompanhar a execução dos currículos dos
-Cursos de Nível Médio ofertados pela Instituição;
-IV - coordenar programas de ensino, metodologias, recursos e instrumentos de
-planejamento em conjunto com o corpo docente e técnico-administrativo;
-V - planejar e acompanhar o sistema de avaliação, processos de transferência e de
-aproveitamento escolar em conjunto com o corpo docente e demais órgãos da Diretoria
-de Ensino;
-VI - manter registro dos instrumentos do processo de ensino-aprendizagem;
-VII - acompanhar a elaboração das adaptações curriculares de discentes, juntamente
-com a Coordenadoria Pedagógica, Coordenadoria de Assuntos Estudantis,
-Coordenadoria de Registros Acadêmicos e os Núcleos;
-VIII - acompanhar e dar suporte às atividades dos Colegiados dos Cursos Técnicos de
-Nível Médio;
-IX - disponibilizar auxílio aos alunos para a realização de projetos de ensino;
-X - acompanhar as pesquisas de natureza técnico-pedagógica relacionadas com
-legislação, organização e funcionamento de sistemas de ensino, processos de
-aprendizagem, administração escolar, métodos e técnicas empregadas;
-XI - auxiliar na elaboração dos horários do ensino médio e educação profissional a cada
-período letivo;
-XII - desempenhar outras atividades correlatas à Coordenadoria, ao cargo ou definidas
-pela legislação e/ou atribuídas pelo superior hierárquico.
-Parágrafo único. Os cursos Técnicos de Nível Médio possuem seus respectivos
-coordenadores designados pelo(a) Diretor(a)-geral do Campus.</t>
-  </si>
-  <si>
-    <t>Coordenadoria de Ensino de Graduação</t>
-  </si>
-  <si>
-    <t>Art. 61. As atividades da Coordenadoria de Ensino de Graduação serão exercidas por um
-servidor efetivo do quadro de pessoal do IFRS designado pelo(a) Diretor(a)-geral do
-Campus.
-18
-Art. 62. Compete à Coordenadoria de Ensino de Graduação as seguintes atribuições:
-I - colaborar com o planejamento e constante aperfeiçoamento da Coordenadoria,
-visando atender as demandas de ensino, pesquisa, extensão e gestão existentes na
-Instituição, racionalizando o uso dos recursos e equipamentos;
-II - elaborar o relatório anual das atividades da Coordenadoria;
-III - planejar o processo de ensino-aprendizagem nos seus aspectos quantitativos e
-qualitativos, com o objetivo de aprimorar e acompanhar a execução dos Projetos
-Pedagógicos dos Cursos de Graduação ofertados pelo Campus Bento Gonçalves e/ou em
-convênio com outras instituições;
-IV - acompanhar a execução dos programas de ensino, metodologias, recursos e
-instrumentos de planejamento em conjunto com o corpo docente e técnico-
-administrativo;
-V - orientar, coordenar e supervisionar as atividades do pessoal docente e técnico-
-administrativo da Coordenadoria, de acordo com a legislação vigente;
-VI - auxiliar na elaboração dos horários do ensino de graduação a cada período letivo;
-VII - acompanhar o sistema de avaliação, processos de transferência e de
-aproveitamento acadêmico em conjunto com o corpo docente e demais órgãos da
-Diretoria de Ensino;
-VIII - acompanhar a elaboração das adaptações curriculares de discentes, juntamente
-com a Coordenadoria Pedagógica, Coordenadoria de Assuntos Estudantis,
-Coordenadoria de Registros Acadêmicos e os Núcleos;
-IX - estudar e sugerir normas, critérios e providências ao(à) Diretor(a) de Ensino sobre a
-execução das atividades de ensino, no seu nível de atuação;
-X - acompanhar e dar suporte aos coordenadores de curso;
-XI - desempenhar outras atividades correlatas à Coordenadoria, ao cargo ou definidas
-pela legislação e/ou atribuídas pelo superior hierárquico.
-Parágrafo único. Os cursos de Graduação possuem seus respectivos coordenadores
-designados pelo(a) Diretor(a)-geral do Campus.</t>
-  </si>
-  <si>
-    <t>Coordenadoria Pedagógica</t>
-  </si>
-  <si>
-    <t>Art. 66. A Coordenadoria Pedagógica é formada por profissionais da educação e possui
-as seguintes atribuições:
-I - colaborar com o planejamento e constante aperfeiçoamento da Coordenadoria,
-visando atender as demandas de ensino, pesquisa, extensão e gestão existentes na
-Instituição, racionalizando o uso dos recursos e equipamentos;
-II - elaborar o relatório anual das atividades da Coordenadoria;
-III - realizar pesquisas de natureza técnico-pedagógica relacionadas com legislação,
-organização e funcionamento de sistemas de ensino, processos de aprendizagem,
-administração escolar, métodos e técnicas empregadas;
-IV - incentivar a implantação de novas metodologias que contemplem temas
-transversais, projetos inter, multi e transdisciplinares;
-V - colaborar com a operacionalização do processo de ensino-aprendizagem;
-VI - realizar o planejamento, a orientação e a supervisão das atividades de ensino e
-aprendizagem, avaliando-as para assegurar a regularidade do desenvolvimento do
-processo educativo;
-VII - colaborar na elaboração de materiais didático-pedagógicos;
-VIII - estimular o intercâmbio de experiências didático-pedagógicas;
-IX - desenvolver atividades de orientação pedagógica aos docentes;
-X - participar de estudos de revisão dos projetos pedagógicos e planos de ensino;
-XI - participar de divulgação de atividades pedagógicas;
-XII – acompanhar a elaboração das adaptações curriculares de discentes, juntamente
-com a Coordenadoria de Assuntos Estudantis, Coordenadoria de Registros Acadêmicos
-e os Núcleos de Ações Afirmativas;
-XIII - participar do processo de recrutamento, seleção, ingresso e qualificação de
-professores substitutos/temporários e discentes na instituição;
-XIV - enviar dados e/ou auxiliar na elaboração do relatório anual da Diretoria de Ensino;
-XV - auxiliar no planejamento e controlar a execução dos programas e projetos de
-ensino, conforme sistemas de informação e normas instituídas;
-XVI - viabilizar as atividades relacionadas a Visitas Técnicas;
-XVII - acompanhar os editais de mobilidade estudantil e enviar as informações para a
-Coordenadoria de Registros Acadêmicos e Diretoria de Ensino;
-22
-XVIII - desempenhar outras atividades correlatas à Coordenadoria, ao cargo ou definidas
-pela legislação e/ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
     <t>Art. 68. A Seção de Estágios está vinculada à Diretoria de Ensino do Campus e possui as
 seguintes atribuições:
 I - colaborar com o planejamento e constante aperfeiçoamento da Seção, visando
@@ -3125,211 +2622,6 @@
 curricular supervisionado, respeitando as atribuições de demais setores competentes.</t>
   </si>
   <si>
-    <t>Seção de Ações de Extensão e de Acompanhamento de Egressos</t>
-  </si>
-  <si>
-    <t>Art. 73. Compete à Seção de Ações de Extensão e de Acompanhamento de Egressos as
-seguintes atribuições:
-I - colaborar com o planejamento e constante aperfeiçoamento da Seção, visando
-atender as demandas de ensino, pesquisa, extensão e gestão existentes na Instituição,
-racionalizando o uso dos recursos e equipamentos;
-II - enviar dados e/ou auxiliar na elaboração do relatório anual da Diretoria de Extensão;
-25
-III - auxiliar no planejamento e controlar a execução das ações de extensão conforme
-sistemas de informação e normas instituídas;
-IV - buscar informações sobre editais para financiamento de projetos e bolsas de
-extensão, tanto de órgãos públicos oficiais quanto de outras entidades nacionais e
-internacionais;
-V - preencher o cadastro e o acompanhamento de egressos através de sistemas
-institucionalizados, subsidiando as Diretorias de Ensino, de Extensão, de Pesquisa, Pós-
-graduação e Inovação, de Administração e de Desenvolvimento Institucional com dados
-e informações;
-VI - desempenhar outras atividades correlatas à Seção, ao cargo ou definidas pela
-legislação e/ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
-    <t>Coordenadoria de Comunicação Social</t>
-  </si>
-  <si>
-    <t>Art. 74. Compete à Coordenadoria de Comunicação Social as seguintes atribuições:
-I - colaborar com o planejamento e constante aperfeiçoamento da Coordenadoria,
-visando atender as demandas de ensino, pesquisa, extensão e gestão existentes na
-Instituição, racionalizando o uso dos recursos e equipamentos;
-II - elaborar o relatório anual das atividades da Coordenadoria;
-III - estudar, planejar, executar e controlar ações de divulgação publicitária e de
-prestação de informações de caráter educativo, informativo e de orientação social,
-estimulando a retroalimentação da comunicação entre a instituição e a comunidade
-externa;
-IV - zelar pela preservação da identidade visual da instituição;
-V - prestar apoio técnico à Diretoria de Extensão na participação em eventos internos e
-externos;
-VI - integrar a Comissão Permanente de Formatura do Campus Bento Gonçalves;
-VII - gerenciar a utilização das salas de Audiosvisuais e do Salão de Atos do Campus Bento
-Gonçalves, bem como zelar pela preservação dos mesmos;
-VIII - instalar, ligar, testar e gerenciar equipamentos de audiovisual;
-IX - prestar apoio técnico na produção de material didático e/ou de divulgação de
-ensino; pesquisa, extensão e gestão que necessitar de recursos audiovisuais;
-X - elaborar o Plano Anual de Comunicação;
-XI - orientar gestores e demais servidores para a consolidação do relacionamento com
-a imprensa;
-XII - produzir releases de interesse institucional e enviá-los à imprensa;
-XIII - gerenciar a alimentação de informações no sítio eletrônico e nas páginas nas redes
-sociais do Campus na internet;
-XIV - presidir a comissão responsável pela edição e publicação do Boletim de Serviços;
-XV - desempenhar outras atividades correlatas à Coordenadoria, ao cargo ou definidas
-pela legislação e/ou atribuídas pelo superior hierárquico.
-26
-§ 1° A execução das atividades da Coordenadoria de Comunicação Social será feita por
-equipe composta minimamente por jornalista, técnicos audiovisuais e demais cargos
-necessários.
-§ 2° As atribuições dos servidores mencionados no § 1º deste artigo serão as previstas
-em cada um de seus cargos, segundo a legislação vigente.</t>
-  </si>
-  <si>
-    <t>Secretaria de Pós-graduação</t>
-  </si>
-  <si>
-    <t>Art. 78. A Secretaria de Pós-graduação é o órgão executivo dos serviços administrativos,
-acadêmicos e técnicos de suporte à pesquisa e à pós-graduação, e a ela compete:
-I - colaborar com o planejamento e constante aperfeiçoamento da Secretaria, visando
-atender as demandas de ensino, pesquisa, extensão e gestão existentes na Instituição,
-racionalizando o uso dos recursos e equipamentos;
-II - colaborar com a proposição e o desenvolvimento dos cursos de pós-graduação lato
-sensu e stricto sensu, em articulação com a Diretoria de Ensino, e supervisioná-los;
-27
-III - atender e dar suporte às coordenações de curso de pós-graduação, professores,
-alunos e público externo;
-IV - divulgar eventos relacionados à pós-graduação;
-V - dar suporte e auxiliar no andamento dos fluxos das propostas e processos de pós-
-graduação em andamento no Campus;
-VI - redigir, receber, classificar, arquivar e expedir documentos, memorandos,
-certificados, diplomas, atestados, declarações, conteúdos programáticos e demais
-documentos da pós-graduação que sejam solicitados;
-VII - efetivar e coordenar as atividades administrativas referentes ao registro acadêmico,
-matrículas, ajustes de matrículas, trancamentos, ajustes de notas, frequência, registros
-de proficiência em língua estrangeira, diplomação e conclusão de cursos de pós-
-graduação;
-VIII - organizar e manter atualizada a coletânea de legislação, resoluções, instruções
-normativas, ofícios e demais documentos;
-IX - arquivar pastas de alunos egressos;
-X - arquivar processos de alunos pós-graduandos;
-XI - dar suporte às coordenações de cursos de pós-graduação do Campus nos processos
-de lançamento de edital para ingresso de alunos, auxiliando na proposição de
-cronogramas, controle de prazos, publicações e homologações;
-XII - juntar documentação relativa à defesa no processo de diplomação do pós-
-graduando, bem como tramitar o processo para registro na Reitoria.
-Parágrafo único. Os assuntos de caráter didático-pedagógico, disciplinar, normas
-regimentais, entre outros de ensino serão abordados, com tomadas de decisão, em
-reunião coletiva com a presença do(a) Diretor(a) de Pesquisa, Pós-Graduação e Inovação
-e de professores, em articulação com as Diretorias de Ensino, de Extensão, de
-Administração e de Desenvolvimento Institucional, Coordenadorias e Seções, quando
-necessário.</t>
-  </si>
-  <si>
-    <t>Seção de Ações de Pesquisa e Inovação</t>
-  </si>
-  <si>
-    <t>Art. 79. A Seção de Ações de Pesquisa e Inovação é responsável por:
-I - colaborar com o planejamento e constante aperfeiçoamento da Seção, visando
-atender as demandas de ensino, pesquisa, extensão e gestão existentes na Instituição,
-racionalizando o uso dos recursos e equipamentos;
-II - enviar dados e/ou auxiliar na elaboração do relatório anual da Diretoria de Pesquisa,
-Pós-graduação e Inovação;
-III - acompanhar os programas e projetos de pesquisas e inovação, integrados ou não,
-com organizações, em todos os níveis e modalidades de ensino, segundo
-regulamentações vigentes;
-IV - estudar e sugerir normas, critérios e providências ao(à) Diretor(a) de Pesquisa, Pós-
-graduação e Inovação sobre a execução das atividades de pesquisa e inovação;
-28
-V - buscar informações sobre editais para financiamento de projetos e bolsas de
-pesquisa, tanto de órgãos públicos oficiais quanto de outras entidades nacionais e
-internacionais;
-VI - participar de fóruns nacionais de pesquisa;
-VII - divulgar e orientar pesquisadores e alunos acerca dos editais, resoluções, instruções
-normativas e documentos técnicos emitidos e publicados pela Pró-reitoria de Pesquisa,
-Pós-graduação e Inovação e Direção-geral;
-VIII - desempenhar outras atividades correlatas à Seção, ao cargo ou definidas pela
-legislação e/ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
-    <t>Seção de Planejamento e Pesquisa Institucional</t>
-  </si>
-  <si>
-    <t>Art. 113. À Seção de Planejamento e Pesquisa Institucional compete:
-I - colaborar com o planejamento e constante aperfeiçoamento da Seção, visando
-atender as demandas de ensino, pesquisa, extensão e gestão existentes na Instituição,
-racionalizando o uso dos recursos e equipamentos;
-II - prover dados e auxiliar na elaboração do relatório anual da Diretoria de
-Desenvolvimento Institucional;
-III - responder aos censos e alimentar outros sistemas de coleta de dados educacionais
-mantidos por órgãos superiores, compilando os dados no âmbito do Campus;
-IV - atualizar, acompanhar e prestar informações referentes aos dados educacionais do
-Campus;
-V - disponibilizar informações para a Comissão Própria de Avaliação (CPA) local;
-VI - fornecer informações acadêmicas para a elaboração do Relatório de Gestão;
-40
-VII - coordenar a elaboração dos Relatórios de Desenvolvimento Institucional para
-Acompanhamento de Curso, em parceria com as coordenações e os colegiados de curso,
-e com a Diretoria de Ensino;
-VIII - auxiliar na elaboração e acompanhamento da execução do planejamento
-institucional e do Plano de Ação, juntamente com as diretorias, por meio de orientações,
-capacitações e uso de ferramentas de gestão apropriadas;
-IX - desempenhar outras atividades correlatas à Seção ou ao cargo, além daquelas
-definidas pela legislação ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
-    <t>Assessoria de Gestão de Projetos e Parcerias</t>
-  </si>
-  <si>
-    <t>Art. 114. A Assessoria de Gestão de Projetos e Parcerias é responsável por:
-I - colaborar com o planejamento e constante aperfeiçoamento da Assessoria, visando
-atender as demandas de ensino, pesquisa, extensão e gestão existentes na Instituição,
-racionalizando o uso dos recursos e equipamentos;
-II - prover dados e auxiliar na elaboração do relatório anual da Diretoria de
-Desenvolvimento Institucional;
-III - auxiliar na elaboração e acompanhamento da execução do planejamento
-institucional, juntamente com as diretorias;
-IV - acompanhar o cumprimento das metas definidas nos planos de acordo do IFRS;
-V - intermediar os trâmites para a realização de parcerias da instituição com outras
-organizações, formalizando-os;
-VI - manter atualizado o cadastro de organizações com as quais o Campus possui
-parcerias;
-VII - auxiliar no planejamento e gestão dos projetos resultantes do PDI, do Plano de
-Ação, de parcerias e projetos institucionais, por meio de orientações, capacitações e uso
-de técnicas apropriadas a cada projeto estabelecido;
-VIII - desempenhar outras atividades correlatas à Assessoria ou ao cargo, além daquelas
-definidas pela legislação ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
-    <t>Regime Disciplinar Do Servidor</t>
-  </si>
-  <si>
-    <t>Art. 149. O regime disciplinar, constando direitos e deveres do corpo docente e do corpo
-técnico-administrativo do Campus, observará as disposições legais, as legislações,
-normas e regulamentos sobre a ordem disciplinar e sanções aplicáveis, bem como os
-recursos cabíveis previstos pela legislação federal.
-48
-Art. 150. A Direção-Geral do Campus que tiver conhecimento de irregularidade no
-âmbito de sua responsabilidade é obrigada a promover a sua imediata apuração,
-mediante sindicância ou processo administrativo disciplinar, assegurando ao servidor
-ampla defesa e contraditório.
-Parágrafo único. Fica facultado ao(à) Diretor(a)-geral encaminhar as denúncias de
-irregularidades à Comissão de Ética para seu parecer.
-Art. 151. Qualquer pessoa poderá, de forma fundamentada, representar contra servidor
-que cometeu ato passível de punição disciplinar junto à Direção-Geral do Campus em
-que o servidor está lotado.</t>
-  </si>
-  <si>
-    <t>Regime Disciplinar Dos Discentes</t>
-  </si>
-  <si>
-    <t>Art. 152. O regime disciplinar do corpo discente é o estabelecido em regulamento
-próprio aprovado pelo Conselho do Campus.
-Art. 153. Qualquer pessoa poderá, de forma fundamentada, representar contra o
-discente que cometeu ato passível de punição disciplinar junto à Diretoria de Ensino do
-Campus.</t>
-  </si>
-  <si>
     <t>Art. 13º A Coordenação de Curso, subordinadas à Direção de Ensino, é
 o órgão responsável pela gestão didático-pedagógica do curso, exercida por
 um docente efetivo do Campus Canoas.
@@ -3339,9 +2631,6 @@
   </si>
   <si>
     <t>Resolução Nº 14 - Regimento Complementar do Campus Canoas - Ano 2018</t>
-  </si>
-  <si>
-    <t>– Do Setor Pedagógico</t>
   </si>
   <si>
     <t>Art. 31º Ao Setor de Pedagógico, subordinado à Coordenadoria de
@@ -3363,9 +2652,6 @@
   </si>
   <si>
     <t>Resolução Nº 23 - Regimento Complementar do Campus Ibirubá - Ano 2025</t>
-  </si>
-  <si>
-    <t>Coordenadoria de Produção Agropecuária</t>
   </si>
   <si>
     <t>Art.46 A Coordenadoria de Produção Agropecuária é um órgão executivo do
@@ -3412,82 +2698,6 @@
 de acordo com a necessidade e evolução da extensão no Campus.
 Art.48 A Coordenadoria de produção agropecuária é composta pela Seção de
 Agroindústria, Seção de Produção Vegetal e Seção de Produção Animal.</t>
-  </si>
-  <si>
-    <t>Seção de Produção Vegetal</t>
-  </si>
-  <si>
-    <t>Art.50 Compete à Seção de Produção Vegetal as seguintes atribuições:
-I. Planejar, executar e acompanhar práticas agrícolas relacionadas à
-semeadura ou plantio, adubação, irrigação, manejo integrado de
-pragas, doenças, plantas daninhas, colheita e pós-colheita;
-II. Orientar e realizar o uso correto, seguindo as recomendações
-técnicas dos insumos (sementes, adubos, defensivos, dentre outros);
-III. Realizar o descarte correto de embalagens de insumos e defensivos
-agrícolas;
-IV. Dar destino correto para óleos usados, filtros e peças obsoletas;
-V. Regular e utilizar máquinas, implementos e equipamentos no setor,
-bem como acompanhar o preparo do solo, pulverizações, plantios,
-colheitas, transporte de produtos, dentre outras operações;
-VI. Fornecer matéria-prima de origem vegetal para merenda escolar e
-para a agroindústria da instituição, quando solicitado;
-VII. Requisitar e acompanhar serviços de manutenção de tratores,
-máquinas, implementos agrícolas e veículos;
-VIII. Elaborar e executar formas de controle de manutenção preventiva de
-máquinas e equipamentos agrícolas;
-IX. Prestar serviços com máquinas e implementos agrícolas para as
-demais seções do Campus, conforme solicitação e pré-agendamento;
-X. Dar suporte técnico para que as aulas teórico-práticas e projetos de
-pesquisa, de ensino e extensão possam ser desenvolvidos atendendo
-o currículo preestabelecido;
-XI. Planejar e requisitar à coordenadoria a compra de materiais,
-equipamentos, insumos e produtos afins, para atender as
-necessidades no desenvolvimento das atividades, com antecedência
-e tempo hábil;
-XII. Elaborar, periodicamente, pareceres e relatórios à Coordenadoria,
-visando subsidiar tomadas de decisões relativas à seção;
-XIII. Comunicar à Agroindústria a disponibilidade de produtos para
-processamento;
-22
-XIV. Orientar e utilizar vestimenta e equipamentos de proteção (EPIs)
-adequados à legislação;
-XV. Zelar pela conservação dos materiais, equipamentos e instalações do
-setor;
-XVI. Desempenhar outras atividades correlatas à seção, ao cargo ou
-definidas pela legislação e/ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
-    <t>Seção de Produção Animal</t>
-  </si>
-  <si>
-    <t>Art.51 Compete à Seção de Produção Animal as seguintes atribuições:
-I. Planejar e realizar o manejo necessário para um bom desempenho
-zootécnico, observando o bem-estar animal;
-II. Elaborar, periodicamente, pareceres e relatórios à Coordenadoria,
-visando subsidiar tomadas de decisões relativas a seção;
-III. Planejar, juntamente à seção de produção vegetal, a implantação e
-condução de pastagens e/ou culturas alternativas para alimentação
-dos animais;
-IV. Planejar e requisitar à coordenadoria a aquisição de materiais,
-equipamentos, medicamentos e produtos afins, para atender as
-necessidades no desenvolvimento das atividades, com antecedência
-e tempo hábil;
-V. Dar suporte técnico para que as aulas teóricos-práticas e projetos de
-pesquisa, de ensino e extensão possam ser desenvolvidos atendendo
-o currículo preestabelecido;
-VI. Zelar pela conservação dos materiais, equipamentos e instalações do
-setor;
-VII. Supervisionar a atividade de ordenha dos animais, observando
-padrões de qualidade e normas técnicas;
-VIII. Orientar e utilizar vestimenta e equipamentos de proteção (EPIs)
-adequados à legislação;
-IX. Fornecer matéria-prima de origem animal para merenda escolar e
-para a agroindústria da instituição, quando solicitado;
-X. Auxiliar na elaboração de documentos relativos à venda ou doação de
-animais;
-XI. Desempenhar outras atividades correlatas à seção, ao cargo ou
-definidas pela legislação e/ou atribuídas pelo superior hierárquico.
-23</t>
   </si>
   <si>
     <t>Núcleo de Ensino a Distância (NEAD)</t>
@@ -4163,14 +3373,6 @@
 eleitos(as) por seus pares para mandato de 2(dois) anos;
 IV – Por 4 (quatro) representantes do segmento discente, eleitos(as) por
 seus pares para mandato de 1 (um) ano.</t>
-  </si>
-  <si>
-    <t>Comissão de Avaliação e Gestão de Ensino, Pesquisa e Extensão (CAGEPE)</t>
-  </si>
-  <si>
-    <t>Art. 93. A Comissão de Avaliação e Gestão de Ensino, Pesquisa e Extensão (CAGEPE) deverá
-auxiliar a Direção de Ensino, a Coordenadoria de Extensão e a Coordenadoria de Pesquisa, Pós-
-graduação e Inovação nas ações inerentes aos processos de ensino, pesquisa e extensão.</t>
   </si>
   <si>
     <t>Comissão Permanente de Licitação</t>
@@ -5367,39 +4569,6 @@
 XVIII - desempenhar outras atividades correlatas ao cargo ou definidas pela legislação vigente e/ou atribuídas pelo superior hierárquico.</t>
   </si>
   <si>
-    <t>Art. 9. O Setor de Comunicação, concebido como sistêmico dentro da unidade por congregar ações que integram as áreas do ensino, da pesquisa e da extensão, é responsável pela comunicação do Campus com seus públicos.
-Parágrafo único. As atividades do Setor de Comunicação serão exercidas por equipe composta por jornalista, técnico audiovisual e demais cargos necessários.
-Art. 10. Ao Setor da Comunicação, subordinado à Direção Geral, compete as seguintes atribuições:
-I. Estudar, planejar, executar e controlar ações de divulgação publicitária e de prestação de informações de caráter educativo, informativo e de orientação social;
-II. Zelar pela preservação da identidade visual da Instituição;
-III. Prestar apoio técnico à Coordenadoria de Extensão na participação em eventos internos e externos;
-IV. Gerenciar a utilização das salas de recursos audiovisuais do Campus;
-V. Instalar, ligar, testar e gerenciar equipamentos de audiovisual;
-VI. Prestar apoio técnico na produção de material didático e/ou de divulgação;
-VII. Elaborar o Plano Anual de Comunicação;
-VIII. Orientar gestores e demais servidores para a consolidação do relacionamento com a imprensa;
-IX. Produzir informativos de interesse institucional e enviá-los à imprensa;
-X. Gerenciar a alimentação de informações no sítio eletrônico e nas páginas nas redes sociais;
-XI. Integrar a Comissão responsável pela edição e publicação do Boletim de Serviços;
-XII. Estabelecer critérios de fixação e controle de cartazes, faixas e murais;
-XIII. Implementar ações provenientes da política de comunicação do IFRS;
-XIV. Participar da Comissão Permanente de Formatura;
-XV. Participar da Comissão Permanente de Seleção do Processo Seletivo;
-XVI. Desempenhar outras atividades correlatas ao setor de comunicação, ao cargo ou definidas pela legislação e/ou atribuídas pelo superior hierárquico.
-Art. 11. Compete ao jornalista:
-I. Promover a divulgação jornalística de eventos por diferentes veículos;
-II. Estabelecer contato com veículos de comunicação e promover a divulgação das ações;
-III. Trabalhar na criação e manutenção de publicações jornalísticas em nível de campus.
-Art. 12. Compete ao Técnico em Audiovisual:
-I. Produzir e editar filmes institucionais em conjunto com o jornalista;
-II. Atuar com equipamentos audiovisuais;
-III. Manejar equipamentos audiovisuais, registrando som, foto e vídeo;
-IV. Zelar pelo cumprimento das normas de uso de imagem;
-V. Manter e conservar os equipamentos;
-VI. Controlar a circulação dos equipamentos;
-VII. Manter organizados os arquivos de imagens e áudio.</t>
-  </si>
-  <si>
     <t>Art. 11. A Coordenadoria de Gestão de Pessoas (CGP) é o órgão responsável por planejar, coordenar, gerir e supervisionar a execução de atividades relacionadas às políticas de gestão de pessoas.
 Art. 12. As atividades da Coordenadoria de Gestão de Pessoas serão exercidas por um servidor efetivo do quadro de pessoal do IFRS designado pelo(a) Diretor(a) Geral do Campus.
 Art. 13. À Coordenadoria de Gestão de Pessoas, subordinada à Direção Geral, compete as seguintes atribuições:
@@ -5696,20 +4865,6 @@
 Art. 57. Os demais espaços de inovação do Campus são vinculados à Coordenadoria de Pesquisa, Pós-graduação e Inovação, com regulamentação própria.</t>
   </si>
   <si>
-    <t>Art. 56. As atividades de Gestão de Extensão serão exercidas por um servidor efetivo do quadro de pessoal do IFRS designado pelo(a) Diretor(a) Geral do Campus.
-Parágrafo único. Compete à Gestão de Extensão, subordinada à Direção Geral, além das competências previstas em legislação vigente e do estabelecido em Estatuto, Regimentos e Regulamentos do IFRS, as atribuições previstas em regulamentação própria aprovada pelo Conselho Superior do IFRS.
-Art. 57. A Coordenadoria de Extensão é composta pelo Setor de Estágios e Egressos, o Núcleo de Ações Afirmativas e o Núcleo de Memória.
-Art. 58. Compete à Coordenadoria de Extensão:
-I – Promover e expandir as ações de extensão, com estreita relação entre ensino e pesquisa;
-II – Viabilizar mecanismos de acesso da sociedade às atividades da Instituição;
-III – Fomentar a participação dos servidores em Editais de extensão;
-IV – Apoiar o desenvolvimento de ações de integração com o mundo do trabalho;
-V – Realizar os encaminhamentos das atividades de estágio curricular;
-VI – Apoiar o desenvolvimento de ações inclusivas vinculadas aos núcleos institucionais, incluindo NAPNE, NEABI, NEPGS, NAC, NEA e NuMem;
-VII – Organizar, divulgar e estimular a participação no evento anual de extensão;
-VIII – Desempenhar as demais atribuições inerentes a essa área.</t>
-  </si>
-  <si>
     <t>Art. 65. As atividades de Gestão da Coordenadoria de Desenvolvimento Institucional serão exercidas por um servidor efetivo do quadro de pessoal do IFRS designado pelo(a) Diretor(a) Geral.
 Parágrafo único. Compete à Gestão de Desenvolvimento Institucional, subordinada à Direção Geral, além das competências previstas em legislação vigente e do estabelecido em Estatuto, Regimentos e Regulamentos do IFRS, as atribuições previstas em regulamentação própria aprovada pelo Conselho Superior do IFRS.
 Art. 66. Compete à Coordenadoria de Desenvolvimento Institucional:
@@ -6051,70 +5206,6 @@
 regimento específico.</t>
   </si>
   <si>
-    <t>Resolução Nº 034 - Regimento Complementar do Campus Bento Gonçalves - Ano 2024
-Art. 56. A Auditoria Interna do Campus Bento Gonçalves integra a Unidade de Auditoria Interna do IFRS (UNAI-IFRS), que está vinculada ao Conselho Superior do IFRS e tem sua estrutura organizada conforme regimento específico.
-§ 1° A auditoria interna do Campus Bento Gonçalves é formada por um Auditor Interno e equipe de apoio sob sua chefia, conforme necessidade.
-§ 2° A auditoria interna do Campus Bento Gonçalves possui subordinação hierárquica à UNAI-IFRS, contudo, administrativamente, está vinculada à Direção-geral do Campus.
-§ 3° As competências do Auditor Interno estão dispostas no regimento da Unidade de Auditoria Interna do IFRS.
-Resolução Nº 23 - Regimento Complementar do Campus Ibirubá - Ano 2025
-Art. 112. As atividades de Auditoria Interna no Campus Ibirubá são exercidas pela Unidade de Auditoria Interna do IFRS (UNAI), que está vinculada ao Conselho Superior do IFRS e possui composição, competências e funcionamento definidos no Regimento Interno da UNAI do IFRS.
-Parágrafo Único. Os Auditores lotados e/ou em exercício no Campus são subordinados ao Auditor-chefe da UNAI.
-Resolução Nº 14 - Regimento Complementar do Campus Canoas - Ano 2018
-Art. 27º O Setor de Auditoria Interna do Campus Canoas integra a Unidade de Auditoria Interna do Instituto Federal de Educação, Ciência e Tecnologia do Rio Grande do Sul – UNAI/IFRS – que está vinculada ao Conselho Superior do IFRS e tem sua estrutura organizada conforme regimento específico.
-Art. 28º A Auditoria Interna do Campus Canoas possui subordinação hierárquica à UNAI/IFRS, administrativamente está vinculada à Direção Geral do Campus.
-Art. 29º As competências do Auditor Interno estão dispostas no Regimento da Unidade de Auditoria Interna do Instituto Federal de Educação, Ciência e Tecnologia do Rio Grande do Sul.</t>
-  </si>
-  <si>
-    <t>Art. X. A Auditoria Interna do Campus integra a Unidade de Auditoria Interna do IFRS (UNAI-IFRS), que está vinculada ao Conselho Superior do IFRS e tem sua estrutura, composição, competências e funcionamento organizados conforme regimento específico. § 1º A Auditoria Interna do Campus é formada por um Auditor Interno e equipe de apoio sob sua chefia, conforme necessidade, sendo os auditores lotados e/ou em exercício no Campus subordinados ao Auditor-chefe da UNAI-IFRS. § 2º A Auditoria Interna do Campus possui subordinação hierárquica à UNAI-IFRS, contudo, administrativamente, está vinculada à Direção Geral do Campus. § 3º As competências do Auditor Interno estão dispostas no Regimento da Unidade de Auditoria Interna do IFRS.</t>
-  </si>
-  <si>
-    <t>Art. X. Ao Setor de Ensino, subordinado à Diretoria de Ensino, compete as seguintes atribuições:
-I - colaborar com o planejamento e constante aperfeiçoamento do setor, visando atender as demandas de ensino, pesquisa, extensão e gestão existentes na Instituição, racionalizando o uso dos recursos e equipamentos;
-II - elaborar, propor e desenvolver projetos de apoio ao ensino, à pesquisa, à extensão e à gestão em consonância com os setores envolvidos;
-III - apoiar as Coordenações de Ensino, Pesquisa e Extensão em atividades técnico-pedagógicas;
-IV - planejar, organizar e divulgar ações relativas às atividades de ensino em todos os níveis;
-V - elaborar e acompanhar, juntamente com a Comissão de Avaliação e Gestão do Ensino (CAGE), o calendário acadêmico para todos os níveis de ensino;
-VI - acompanhar a elaboração dos horários dos cursos regulares ofertados no Campus juntamente com os Coordenadores de Curso;
-VII - coordenar, acompanhar e avaliar o desenvolvimento do processo de ensino-aprendizagem;
-VIII - acompanhar, juntamente com a Direção de Ensino, Setor Pedagógico, Assistência Estudantil, Coordenação de Curso, docentes e representação estudantil, reuniões de Conselhos de Classe;
-IX - acompanhar a elaboração e o arquivamento de planos de ensino e diários de classe;
-X - verificar e emitir atestados de docência;
-XI - analisar e deferir requerimentos acerca de justificativas e/ou abono de faltas, bem como dos exercícios domiciliares dos estudantes;
-XII - gerenciar, juntamente com a CAGE, o planejamento, a divulgação, a execução e avaliação dos Editais vinculados ao Ensino;
-XIII - viabilizar ações de Permanência e Êxito dos estudantes;
-XIV - garantir espaços para a realização de atividades de Formação Continuada dos servidores, prevendo a participação dos Núcleos de Ações Afirmativas;
-XV - promover ações que visem ao compartilhamento de conhecimentos e à integração da comunidade acadêmica, tais como Seminários, Mostras de Trabalhos, Oficinas e Simpósios;
-XVI - acompanhar as solicitações de viagens de estudo e/ou viagens técnicas junto às Coordenações de Curso;
-XVII - implementar programas de tecnologia educacional;
-XVIII - participar de estudos de revisão de currículo e programas de ensino;
-XIX - desempenhar outras atividades correlatas ao setor, ao cargo ou definidas pela legislação e/ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
-    <t>Art. X. O Setor Pedagógico, subordinado à Diretoria de Ensino, tem a função de atuar de forma integrada no acompanhamento, na assessoria e na mediação do trabalho pedagógico, articulando a ação educativa à Proposta Pedagógica da Instituição, viabilizando o trabalho coletivo e contribuindo para a qualificação das relações no processo educativo, bem como na formação humana, técnica e científica.
-Art. X. Compete ao Setor Pedagógico as seguintes atribuições:
-I - orientar e acompanhar ocorrências relativas ao andamento das aulas, à preservação do patrimônio, ao cumprimento das normas, aos aspectos disciplinares e ao bem-estar dos alunos;
-II - acompanhar e supervisionar a entrada, permanência, saída e demais atividades do corpo discente;
-III - encaminhar o aluno, em caso de emergência, ao serviço médico ou odontológico, informando os familiares;
-IV - contribuir com a comunicação dos assuntos referentes ao Setor de forma eficiente e integrada com os demais setores do Campus;
-V - participar na elaboração e publicizar as normas internas do Campus à toda a comunidade institucional;
-VI - orientar docentes e discentes sobre as atividades e atribuições pertinentes ao Setor Pedagógico;
-VII - coordenar, acompanhar e orientar o planejamento das atividades pedagógicas;
-VIII - participar da elaboração, execução e avaliação do Projeto Pedagógico Institucional e dos Projetos Pedagógicos dos Cursos;
-IX - acompanhar e mediar as práticas pedagógicas no que se refere ao processo ensino-aprendizagem;
-X - mediar a elaboração, a execução e o arquivamento dos planos de ensino em todos os níveis de ensino;
-XI - orientar e monitorar a finalização e o arquivamento dos diários de classe em todos os níveis de ensino;
-XII - acompanhar a elaboração dos programas de adaptação de currículo, atividades de reforço escolar e estudos de recuperação;
-XIII - discutir, propor e analisar resultados da ação pedagógica, visando à construção coletiva de alternativas para o êxito do processo ensino-aprendizagem e à promoção do desenvolvimento integral do educando;
-XIV - acompanhar as relações entre instituição e família dos estudantes, através de encontros individuais e coletivos, tendo em vista a construção conjunta de propostas que levem à melhoria do processo ensino-aprendizagem;
-XV - organizar e orientar ações relativas à Progressão Parcial;
-XVI - acompanhar substituições e reposições de aulas dos componentes curriculares por motivos previstos em legislação;
-XVII - informar ao Núcleo de Educação a Distância (NEAD) do Campus a relação de docentes e componentes curriculares para cadastramento no Ambiente Virtual de Ensino e Aprendizagem;
-XVIII - desempenhar outras atividades correlatas ou definidas pela legislação e/ou atribuídas pelo superior hierárquico.</t>
-  </si>
-  <si>
-    <t>– Das Coordenadorias de Cursos (Ou deixamos separado igual Bento)</t>
-  </si>
-  <si>
     <t>Subordinação</t>
   </si>
   <si>
@@ -6138,14 +5229,193 @@
     <t>Resolução Nº 20 - Regimento Complementar do Campus Erechim - Ano 2024, Art. 26º.</t>
   </si>
   <si>
-    <t>Setor transferido para a Reitoria</t>
+    <t xml:space="preserve">Coordenadoria de Comunicação </t>
+  </si>
+  <si>
+    <t>Ao setor de Gestão e Fiscalização de Contratos, subordinado a Direção de Administração e Planejamento, compete:
+I – acompanhar a execução dos contratos administrativos do campus;
+II – orientar e apoiar os fiscais de contratos do campus;
+III – acompanhar prazos de vigência, prorrogação, reajuste e renovação contratual;
+IV – instruir processos e procedimentos relativos à gestão contratual;
+V – manter atualizados os registros e documentos dos contratos;
+VI – comunicar ocorrências na execução contratual aos setores e autoridades competentes;
+VII – subsidiar a tomada de decisão em matéria contratual;
+VIII – atuar em articulação com os demais setores envolvidos na contratação e execução contratual;
+IX – zelar pelo cumprimento da legislação e das normas aplicáveis aos contratos administrativos;
+X – exercer outras atribuições correlatas à sua área de atuação.</t>
+  </si>
+  <si>
+    <t>Coordenação Agropecuária</t>
+  </si>
+  <si>
+    <t>Setor de Comunicação (Excluido - Vamos criar a Coordenadoria de Comunicação)</t>
+  </si>
+  <si>
+    <t>Art. 74. Compete à Coordenadoria de Comunicação  as seguintes atribuições:
+I - colaborar com o planejamento e constante aperfeiçoamento da Coordenadoria,
+visando atender as demandas de ensino, pesquisa, extensão e gestão existentes na
+Instituição, racionalizando o uso dos recursos e equipamentos;
+II - elaborar o relatório anual das atividades da Coordenadoria;
+III - estudar, planejar, executar e controlar ações de divulgação publicitária e de
+prestação de informações de caráter educativo, informativo e de orientação social,
+estimulando a retroalimentação da comunicação entre a instituição e a comunidade
+externa;
+IV - zelar pela preservação da identidade visual da instituição;
+V - prestar apoio técnico à coordenação de Extensão na participação em eventos internos e
+externos;
+VI - integrar a Comissão Permanente de Formatura do Campus Vacaria;
+VII - instalar, ligar, testar e gerenciar equipamentos de audiovisual;
+IX - prestar apoio técnico na produção de material didático e/ou de divulgação de
+ensino; pesquisa, extensão e gestão que necessitar de recursos audiovisuais;
+X - elaborar o Plano Anual de Comunicação;
+XI - orientar gestores e demais servidores para a consolidação do relacionamento com
+a imprensa;
+XII - produzir releases de interesse institucional e enviá-los à imprensa;
+XIII - gerenciar a alimentação de informações no sítio eletrônico e nas páginas nas redes
+sociais do Campus na internet;
+XIV - presidir a comissão responsável pela edição e publicação do Boletim de Serviços;
+XV - desempenhar outras atividades correlatas à Coordenadoria, ao cargo ou definidas
+pela legislação e/ou atribuídas pelo superior hierárquico.
+26
+§ 1° A execução das atividades da Coordenadoria de Comunicação será feita por
+equipe composta minimamente por jornalista, técnicos audiovisuais e demais cargos
+necessários.
+§ 2° As atribuições dos servidores mencionados no § 1º deste artigo serão as previstas
+em cada um de seus cargos, segundo a legislação vigente.</t>
+  </si>
+  <si>
+    <t>Texto Adaptado da - Resolução Nº 034 - Regimento Complementar do Campus Bento Gonçalves - Ano 2024</t>
+  </si>
+  <si>
+    <t>"Art. XX. Compete à Coordenação de Extensão, além das competências previstas no Regimento Geral e na legislação vigente, as seguintes atribuições: I - Planejar, promover e expandir as ações de extensão de forma integrada ao ensino e à pesquisa, visando à relevância social, cultural e de base solidária; II - Viabilizar mecanismos de acesso da sociedade às atividades da Instituição e fomentar a integração com o mundo do trabalho e o empreendedorismo; III - Prospectar editais e orientar a participação de servidores em chamadas para captação de recursos e bolsas de extensão; IV - Gerenciar e fiscalizar as atividades de estágio curricular e o acompanhamento de egressos por meio de sistemas institucionalizados; V - Prestar apoio técnico e institucional às ações inclusivas e aos núcleos vinculados (NAPNE, NEABI, NEPGS, NAC, NEA, NuMem e Ações Afirmativas); VI - Organizar, divulgar e estimular a participação da comunidade acadêmica em eventos anuais de ensino, pesquisa e extensão; VII - Elaborar relatórios de gestão, gerir sistemas de informação e zelar pela utilização racional dos recursos e equipamentos da área; VIII - Desempenhar outras atividades correlatas à gestão da extensão ou atribuídas pelo superior hierárquico."</t>
+  </si>
+  <si>
+    <t>DA COORDENADORIA AGROPECUÁRIA
+Art. 1º A Coordenadoria Agropecuária é um órgão executivo do Campus, subordinado à Diretoria de Ensino, sendo gerido por um coordenador nomeado pelo Diretor-Geral.
+Art. 2º Compete à Coordenadoria Agropecuária e ao seu corpo técnico:
+I. Criar mecanismos de articulação permanente entre produção, ensino, pesquisa e extensão, visando o aperfeiçoamento constante do setor;
+II. Planejar, orientar e realizar a programação anual das atividades e projetos de produção agropecuária do Campus;
+III. Fiscalizar a produção e supervisionar tecnicamente os processos produtivos em todas as áreas do setor;
+IV. Desenvolver, criar e adaptar tecnologias aplicadas à produção agropecuária;
+V. Zelar pela preservação ambiental, recomendando e realizando o destino correto de embalagens de agrotóxicos e resíduos;
+VI. Verificar e manter a infraestrutura, máquinas, instalações e equipamentos, informando a necessidade de novos insumos ou manutenções;
+VII. Conduzir experimentos de pesquisa e apoiar o desenvolvimento de projetos científicos;
+VIII. Receber e coordenar o atendimento às demandas de aulas práticas e projetos pedagógicos dos docentes;
+IX. Avaliar a viabilidade pedagógica, técnica, econômica, ambiental e social da produção a ser executada;
+X. Controlar a comercialização dos produtos produzidos no Setor Agropecuário;
+XI. Elaborar relatórios de prestação de contas das atividades e da produção para as instâncias superiores;
+XII. Organizar e fiscalizar as escalas de trabalho e o acompanhamento do setor durante finais de semana, férias e feriados;
+XIII. Disseminar e fomentar práticas de produção orgânica e o cumprimento de normas técnicas vigentes;
+XIV. Zelar pela segurança do trabalho, utilizando obrigatoriamente Equipamentos de Proteção Individual (EPI) e recursos de informática necessários;
+XV. Analisar o registro de frequência dos servidores sob sua competência;
+XVI. Participar ativamente das atividades e eventos programados pelo Campus;
+XVII. Desempenhar outras tarefas de mesma natureza, atividades correlatas ou definidas pela legislação e instâncias superiores.
+Parágrafo único. Compete ao Coordenador Agropecuário zelar para que todas as atribuições descritas neste artigo sejam cumpridas, podendo propor a criação de novas seções conforme a necessidade e evolução das atividades do Campus.</t>
+  </si>
+  <si>
+    <t>Criou-se a coordenadoria.</t>
+  </si>
+  <si>
+    <t>Art. XXº A Coordenação de Curso, subordinadas à coordenação de Ensino, é
+o órgão responsável pela gestão didático-pedagógica do curso, exercida por
+um docente efetivo do Campus.
+Parágrafo único. As atribuições estão estabelecidas por meio de
+Resolução do Conselho Superior do IFRS.</t>
+  </si>
+  <si>
+    <t>Criou-se o setor pedagógico.</t>
+  </si>
+  <si>
+    <t>DO SETOR PEDAGÓGICO
+Art. 1º O Setor Pedagógico, subordinado à Coordenação de Ensino, tem a função de atuar de forma integrada no acompanhamento, na assessoria e na mediação do trabalho pedagógico e administrativo-educacional, articulando a ação educativa à Proposta Pedagógica da Instituição, viabilizando o trabalho coletivo e contribuindo para a qualificação das relações no processo educativo, bem como na formação humana, técnica e científica.
+Art. 2º Compete ao Setor Pedagógico as seguintes atribuições:
+I. Planejamento e Aperfeiçoamento: Colaborar com o planejamento e constante aperfeiçoamento do setor, visando atender as demandas de ensino, pesquisa, extensão e gestão, racionalizando o uso de recursos e equipamentos;
+II. Apoio e Projetos: Elaborar, propor e desenvolver projetos de apoio ao ensino, à pesquisa, à extensão e à gestão, prestando assessoria técnico-pedagógica às coordenações de curso e demais setores;
+III. Documentação Institucional: Participar da elaboração, execução e avaliação do Projeto Pedagógico Institucional (PPI), dos Projetos Pedagógicos dos Cursos (PPC) e dos estudos de revisão de currículo;
+IV. Calendário e Horários: Elaborar e acompanhar o calendário acadêmico junto à Comissão de Avaliação e Gestão do Ensino (CAGE), bem como coordenar a elaboração dos horários dos cursos regulares;
+V. Gestão de Planos e Diários: Mediar a elaboração, a execução, o monitoramento e o arquivamento dos planos de ensino e diários de classe em todos os níveis de ensino;
+VI. Processo Ensino-Aprendizagem: Coordenar, acompanhar e mediar as práticas pedagógicas e os resultados da ação educativa, visando à construção de alternativas para o êxito do processo e o desenvolvimento integral do educando;
+VII. Conselhos de Classe: Organizar e acompanhar as reuniões de Conselhos de Classe, articulando a participação da Direção de Ensino, coordenações, docentes e representação estudantil;
+VIII. Permanência e Êxito: Viabilizar ações de permanência e êxito dos estudantes e gerenciar, junto à CAGE, o planejamento e execução de editais vinculados ao ensino;
+IX. Acompanhamento Discente e Disciplinar: Orientar e acompanhar a entrada, permanência e saída dos alunos, zelando pela preservação do patrimônio, cumprimento das normas internas, aspectos disciplinares e bem-estar geral;
+X. Atendimento de Emergência: Encaminhar o aluno, em caso de necessidade, ao serviço médico ou odontológico, garantindo a imediata comunicação aos familiares;
+XI. Relação Instituição-Família: Acompanhar as relações entre a instituição e as famílias dos estudantes por meio de atendimentos individuais ou coletivos, visando a melhoria do processo educativo;
+XII. Ajustes Curriculares: Organizar e acompanhar programas de adaptação de currículo, atividades de reforço, estudos de recuperação, progressão parcial e substituições/reposições de aulas conforme a legislação;
+XIII. Análise de Requerimentos: Analisar e deferir requerimentos sobre justificativas de faltas, abonos e exercícios domiciliares, além de verificar e emitir atestados de docência;
+XIV. Formação e Eventos: Garantir espaços para formação continuada dos servidores e promover eventos de integração acadêmica, como seminários, mostras, oficinas e simpósios;
+XV. Tecnologia Educacional: Implementar programas de tecnologia educacional e articular junto ao Núcleo de Educação a Distância (NEAD) o cadastramento de docentes e componentes em ambientes virtuais;
+XVI. Viagens Técnicas: Acompanhar e processar as solicitações de viagens de estudo e visitas técnicas junto às Coordenações de Curso;
+XVII. Comunicação e Normatização: Publicizar as normas internas e orientar a comunidade acadêmica sobre as atribuições e fluxos do setor de forma eficiente e integrada;
+XVIII. Atividades Correlatas: Desempenhar outras tarefas de mesma natureza, atividades correlatas ou definidas pela legislação e instâncias superiores.</t>
+  </si>
+  <si>
+    <t>Compete à Coordenadoria de Licitações e Contratos:
+I - colaborar com o planejamento e constante aperfeiçoamento da unidade, visando atender as demandas de ensino, pesquisa, extensão e gestão, racionalizando o uso de recursos;
+II - elaborar o relatório anual de atividades;
+III - supervisionar e coordenar as atividades relacionadas aos Setores de Licitações e de Contratos;
+IV - planejar e gerenciar os processos de compras, serviços e contratos em conjunto com a Direção de Administração;
+V - gerir o planejamento anual de necessidades por meio de ações integradas com os setores requisitantes;
+VI - operacionalizar processos licitatórios, leilões e convênios que impliquem movimentação financeira;
+VII - proceder ao lançamento de itens, cronogramas e documentos nos Sistemas Federais de Administração e sistemas institucionais;
+VIII - orientar e padronizar os procedimentos de aquisição de materiais e contratação de serviços;
+IX - executar procedimentos administrativos junto aos fornecedores para estabelecer prazos e condições de entrega;
+X - abrir e conduzir processos administrativos de penalização referentes a processos com ou sem termo de contrato assinado;
+XI - analisar o registro de frequência dos servidores sob sua competência;
+XII - desempenhar outras atividades correlatas atribuídas pelo superior hierárquico ou pela legislação.</t>
+  </si>
+  <si>
+    <t>Art. 40. A Coordenadoria de Ensino, de forma articulada com a Diretoria de Ensino é o órgão
+responsável por planejar, coordenar, executar, acompanhar e avaliar as políticas educacionais e
+diretrizes de ensino no Campus.
+Art. 41. As atividades da Coordenadoria de Ensino serão exercidas por um servidor efetivo do
+quadro de pessoal do IFRS designado pelo(a) Diretor(a) Geral do Campus.
+Art. 42. À Coordenadoria de Ensino, subordinada à Diretoria de Ensino, compete as seguintes
+atribuições:
+I. Colaborar com o planejamento e constante aperfeiçoamento da Coordenadoria, visando
+atender as demandas de ensino, pesquisa, extensão e gestão existentes na Instituição,
+racionalizando o uso dos recursos e equipamentos;
+II. Planejar, acompanhar e avaliar a proposta pedagógica institucional, nos diferentes níveis
+de ensino oferecidos aos discentes;
+III. Acompanhar o planejamento e a execução dos processos de ensino e aprendizagem;
+IV. Acompanhar a elaboração das propostas pedagógicas;
+V. Encaminhar para aprovação do Conselho de Campus os projetos pedagógicos de cursos
+de Ensino Médio;
+VI. Encaminhar para aprovação no Conselho de Campus as normas de utilização dos espaços
+destinados ao ensino;
+VII. Supervisionar os diários de classe dos componentes curriculares de todos os níveis de
+ensino ofertados pelo campus, junto aos professores e acompanhar sua manutenção, bem como
+os registros de rendimento acadêmico dos estudantes;
+VIII. Elaborar e coordenar a publicação de editais relativos a monitorias, promovendo a gestão
+administrativa, incluindo inscrições, controle de frequência e certificação;
+IX. Elaborar quadro de horários;
+X. Organizar os conselhos de classe;
+XI. Propor atividades de capacitação aos Docentes e Técnicos Administrativos em Educação;
+XII. Responder pelo Diretor de Ensino na sua ausência ou impedimento;
+XIII. Desempenhar outras atividades correlatas à Coordenadoria de Ensino, ao cargo ou
+definidas pela legislação e/ou atribuídas pelo superior hierárquico.
+Das Coorde nadorias de Cursos
+Art. 43. As atividades das Coordenadorias de Cursos, subordinadas à Coordenadoria de Ensino,
+serão exercidas por servidores efetivos do quadro de pessoal do IFRS, eleitos pelo respectivo
+colegiado de curso e nomeados pelo(a) Diretor(a) Geral de Campus.
+Parágrafo único. Às Coordenadorias de Cursos compete a gestão didático-pedagógica dos cursos,
+tendo suas atribuições regulamentadas em Regimento próprio aprovado pelo Conselho Superior
+do IFRS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coordenadorias de Cursos </t>
+  </si>
+  <si>
+    <t>Setor Pedagógico</t>
+  </si>
+  <si>
+    <t>Comissão Integrada de Ensino, Pesquisa e Extensão (CIEPE)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6155,14 +5425,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u val="double"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -6196,9 +5458,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -6207,10 +5469,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6516,7 +5776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="84.5703125" customWidth="1"/>
@@ -6530,7 +5790,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>239</v>
+        <v>196</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -6547,7 +5807,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>240</v>
+        <v>197</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
@@ -6556,7 +5816,7 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>193</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -6570,7 +5830,7 @@
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>194</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -6578,7 +5838,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>240</v>
+        <v>197</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -6587,7 +5847,7 @@
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -6604,75 +5864,75 @@
         <v>15</v>
       </c>
       <c r="E5" t="s">
-        <v>196</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E6" t="s">
-        <v>197</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>198</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>199</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>200</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -6680,305 +5940,322 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="E10" t="s">
-        <v>201</v>
+        <v>165</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E11" t="s">
-        <v>202</v>
+        <v>166</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
-      </c>
-      <c r="E12" t="s">
-        <v>203</v>
+        <v>25</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="E13" t="s">
-        <v>204</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>205</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="E15" t="s">
-        <v>206</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
         <v>47</v>
       </c>
-      <c r="C16" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" t="s">
-        <v>58</v>
-      </c>
       <c r="E16" t="s">
-        <v>207</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E17" t="s">
-        <v>208</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="E18" t="s">
-        <v>63</v>
+        <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
-      </c>
-      <c r="C19" t="s">
-        <v>65</v>
+        <v>45</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>214</v>
       </c>
       <c r="D19" t="s">
-        <v>66</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>236</v>
+        <v>55</v>
+      </c>
+      <c r="E19" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="D20" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="E20" t="s">
-        <v>209</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C21" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D21" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E21" t="s">
-        <v>210</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B22" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="C22" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="E22" t="s">
-        <v>211</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B23" t="s">
         <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="D23" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E23" t="s">
-        <v>212</v>
+        <v>174</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B24" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" t="s">
         <v>75</v>
       </c>
-      <c r="C24" t="s">
-        <v>79</v>
-      </c>
-      <c r="D24" t="s">
-        <v>100</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>80</v>
-      </c>
-      <c r="B25" t="s">
-        <v>7</v>
-      </c>
-      <c r="C25" t="s">
-        <v>81</v>
-      </c>
       <c r="D25" t="s">
-        <v>82</v>
-      </c>
-      <c r="E25" t="s">
-        <v>213</v>
+        <v>88</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B26" t="s">
-        <v>80</v>
+        <v>7</v>
       </c>
       <c r="C26" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="D26" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="E26" t="s">
-        <v>214</v>
+        <v>175</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B27" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" t="s">
+        <v>80</v>
+      </c>
+      <c r="D27" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" t="s">
         <v>83</v>
       </c>
-      <c r="C27" t="s">
-        <v>87</v>
-      </c>
-      <c r="D27" t="s">
-        <v>88</v>
-      </c>
-      <c r="E27" t="s">
-        <v>215</v>
+      <c r="D28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -6988,13 +6265,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE40C40-B396-416D-A3C3-A5E69DAF0F21}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="62.28515625" customWidth="1"/>
     <col min="2" max="2" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7008,60 +6286,40 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>25</v>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>204</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>244</v>
+        <v>209</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>28</v>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="D3" t="s">
-        <v>244</v>
+        <v>209</v>
+      </c>
+      <c r="E3" t="s">
+        <v>173</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>31</v>
+    <row r="4" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="D4" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" t="s">
-        <v>244</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -7071,7 +6329,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="91.85546875" customWidth="1"/>
@@ -7083,277 +6341,101 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B1" t="s">
-        <v>239</v>
+        <v>196</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5" t="s">
         <v>92</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="D2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E2" t="s">
-        <v>235</v>
+      <c r="E5" s="2" t="s">
+        <v>208</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" t="s">
-        <v>95</v>
-      </c>
-      <c r="D3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>198</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" t="s">
-        <v>102</v>
+        <v>20</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="D6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>103</v>
-      </c>
-      <c r="B7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" t="s">
-        <v>104</v>
-      </c>
-      <c r="D7" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>105</v>
-      </c>
-      <c r="B8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" t="s">
-        <v>106</v>
-      </c>
-      <c r="D8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>107</v>
-      </c>
-      <c r="B9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" t="s">
-        <v>108</v>
-      </c>
-      <c r="D9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>109</v>
-      </c>
-      <c r="B10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C10" t="s">
-        <v>110</v>
-      </c>
-      <c r="D10" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>111</v>
-      </c>
-      <c r="B11" t="s">
-        <v>240</v>
-      </c>
-      <c r="C11" t="s">
-        <v>112</v>
-      </c>
-      <c r="D11" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>113</v>
-      </c>
-      <c r="B12" t="s">
-        <v>240</v>
-      </c>
-      <c r="C12" t="s">
-        <v>114</v>
-      </c>
-      <c r="D12" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>115</v>
-      </c>
-      <c r="B13" t="s">
-        <v>240</v>
-      </c>
-      <c r="C13" t="s">
-        <v>116</v>
-      </c>
-      <c r="D13" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>238</v>
-      </c>
-      <c r="B14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" t="s">
-        <v>117</v>
-      </c>
-      <c r="D14" t="s">
-        <v>118</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>119</v>
-      </c>
-      <c r="B15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" t="s">
-        <v>120</v>
-      </c>
-      <c r="D15" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>122</v>
-      </c>
-      <c r="B16" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="D16" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>124</v>
-      </c>
-      <c r="B17" t="s">
-        <v>122</v>
-      </c>
-      <c r="C17" t="s">
-        <v>125</v>
-      </c>
-      <c r="D17" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>126</v>
-      </c>
-      <c r="B18" t="s">
-        <v>122</v>
-      </c>
-      <c r="C18" t="s">
-        <v>127</v>
-      </c>
-      <c r="D18" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="B19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="D19" t="s">
-        <v>243</v>
+        <v>200</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -7387,338 +6469,330 @@
     </row>
     <row r="2" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
+        <v>95</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>216</v>
+        <v>151</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>96</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>217</v>
+        <v>98</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>186</v>
+        <v>150</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>99</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>218</v>
+        <v>149</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>134</v>
+        <v>100</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>136</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>219</v>
+        <v>102</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>137</v>
+        <v>103</v>
       </c>
       <c r="B6" t="s">
-        <v>138</v>
+        <v>104</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>220</v>
+        <v>153</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>139</v>
+        <v>105</v>
       </c>
       <c r="B7" t="s">
-        <v>140</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>141</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>221</v>
+        <v>107</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>142</v>
+        <v>108</v>
       </c>
       <c r="B8" t="s">
-        <v>143</v>
+        <v>109</v>
       </c>
       <c r="C8" t="s">
-        <v>144</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>222</v>
+        <v>110</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>145</v>
-      </c>
-      <c r="B9" t="s">
-        <v>146</v>
-      </c>
-      <c r="C9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>146</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>147</v>
+        <v>111</v>
       </c>
       <c r="B10" t="s">
-        <v>148</v>
+        <v>112</v>
       </c>
       <c r="C10" t="s">
-        <v>149</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>223</v>
+        <v>113</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>150</v>
+        <v>114</v>
       </c>
       <c r="B11" t="s">
-        <v>151</v>
+        <v>115</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>224</v>
+        <v>155</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>152</v>
+        <v>116</v>
       </c>
       <c r="B12" t="s">
-        <v>153</v>
+        <v>117</v>
       </c>
       <c r="C12" t="s">
-        <v>154</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>225</v>
+        <v>118</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
       <c r="B13" t="s">
-        <v>156</v>
+        <v>120</v>
       </c>
       <c r="C13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>226</v>
+        <v>121</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>158</v>
+        <v>122</v>
       </c>
       <c r="B14" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
       <c r="C14" t="s">
-        <v>160</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>227</v>
+        <v>124</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>161</v>
+        <v>125</v>
       </c>
       <c r="B15" t="s">
-        <v>162</v>
+        <v>126</v>
       </c>
       <c r="C15" t="s">
-        <v>163</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>228</v>
+        <v>127</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>164</v>
+        <v>128</v>
       </c>
       <c r="B16" t="s">
-        <v>165</v>
+        <v>129</v>
       </c>
       <c r="C16" t="s">
-        <v>166</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>229</v>
+        <v>130</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s">
-        <v>168</v>
+        <v>132</v>
       </c>
       <c r="C17" t="s">
-        <v>169</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>230</v>
+        <v>133</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>170</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>171</v>
+        <v>135</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>171</v>
+        <v>28</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
       <c r="B19" t="s">
-        <v>173</v>
+        <v>137</v>
       </c>
       <c r="C19" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>173</v>
+        <v>28</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>174</v>
+        <v>138</v>
       </c>
       <c r="B20" t="s">
-        <v>175</v>
+        <v>139</v>
       </c>
       <c r="C20" t="s">
-        <v>176</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>231</v>
+        <v>140</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>178</v>
+        <v>142</v>
       </c>
       <c r="B21" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="C21" t="s">
-        <v>179</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>179</v>
+        <v>143</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>180</v>
+        <v>144</v>
       </c>
       <c r="B22" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>188</v>
+        <v>152</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="B23" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>190</v>
+        <v>154</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>182</v>
+        <v>146</v>
       </c>
       <c r="B24" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="C24" t="s">
-        <v>183</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>233</v>
+        <v>147</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>184</v>
+        <v>148</v>
       </c>
       <c r="B25" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>192</v>
+        <v>156</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>